<commit_message>
Add CAT TO question banks and competency mapping for teachers.
Teachers can map Technical Orders onto skills and draft a 20+ item bank from the SPA, then promote reviewed items into the live quiz.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/EdVidura_Requirements_CrossCheck.xlsx
+++ b/docs/EdVidura_Requirements_CrossCheck.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
-          <t>Now (27 Oct 2026)</t>
+          <t>Now (28 Oct 2026)</t>
         </is>
       </c>
       <c r="I1" s="8" t="inlineStr">
@@ -804,19 +804,19 @@
           <t>Noisy LRS activity heatmap (date x learner)</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>No heatmap in analytics templates or modules</t>
+          <t>GET /api/v1/app/analytics learner_heatmap is dates × learners from all xAPI verbs; Diagnostics heatmaps tab renders the live grid</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Build heatmap from xAPI statement counts</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -826,10 +826,14 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr"/>
+          <t>Live noisy LRS date×learner heatmap on Diagnostics</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1035,19 +1039,19 @@
           <t>Per-student time series at day/week/month/quarter, eight charts</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>No granularity controls or per-student time series</t>
+          <t>GET /api/v1/app/analytics time_series: activity + quiz % at day/week/month/quarter (8 charts); Diagnostics has CSS bars + learner picker</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Build aggregation at four granularities and per-student charts</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1057,10 +1061,14 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr"/>
+          <t>Live 8-chart per-student time series on Diagnostics</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1219,19 +1227,19 @@
           <t>Test bank generation (100+ questions)</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Generation creates drafts per request; no bulk bank of 100+ with review workflow</t>
+          <t>POST /api/v1/app/quiz/bank/generate drafts 100+ items with review_status; teacher approves then promote into live quiz</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Add bulk generation and bank management</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1241,10 +1249,14 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr"/>
+          <t>Live 100+ test bank generate + review on Checkpoint</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#quiz</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1262,19 +1274,19 @@
           <t>Assessment export to PDF and Markdown</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>No PDF or Markdown assessment export found</t>
+          <t>GET /api/v1/app/quiz/export format=md|pdf; SPA Export menu and /teacher/quiz/export.md|.pdf download Markdown and printable PDF</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Add export of a quiz or bank to PDF and Markdown</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1284,10 +1296,14 @@
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="inlineStr"/>
+          <t>Live PDF and Markdown assessment export</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#quiz</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1540,19 +1556,19 @@
           <t>LTI group services</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>No group services code; 'group' hits in the repository are unrelated</t>
+          <t>LTI-GS claim on launch; lti_context_groups + group_assignments; local groups when Moodle GS is off; SPA gradebook + /lti-integration</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Implement LTI group services</t>
+          <t>Moodle must enable Group Services for LMS-native groups</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1562,10 +1578,14 @@
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr"/>
+          <t>Live group assignments on Moodle connection + Gradebook</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/lti-integration</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1583,19 +1603,19 @@
           <t>AI essay grading (LLM/RAG compared with instructor answer)</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>No essay grading; only an academic-integrity pattern</t>
+          <t>grade_essay_against_instructor compares student text to instructor answer + RAG chunks; teacher AI form and POST /quiz/essay-grade; never AGS</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Build essay grader and rubric comparison</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1605,10 +1625,14 @@
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr"/>
+          <t>Live essay grade vs instructor answer on Gradebook</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-results</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1908,19 +1932,19 @@
           <t>Group-based assignments (group services)</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Group assignments gate graded quiz GET/POST (403 not_assigned) for learners outside the assigned group; staff bypass; SPA Checkpoint shows the group</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>As AI Assessment F-11</t>
+          <t>Moodle GS HTTP fetch optional</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1930,10 +1954,14 @@
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I26" s="12" t="inlineStr"/>
+          <t>Live group-gated quiz on Checkpoint + /lti-integration</t>
+        </is>
+      </c>
+      <c r="I26" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/lti-integration</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2092,19 +2120,19 @@
           <t>User assignment dashboard API</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>No assignments API for external applications</t>
+          <t>GET /api/v1/xapi/assignments and GET /api/v1/app/assignments return group assignments + per-learner quota</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Build the API</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2114,10 +2142,14 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I30" s="12" t="inlineStr"/>
+          <t>Live assignment dashboard on Diagnostics xAPI tab</t>
+        </is>
+      </c>
+      <c r="I30" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2135,19 +2167,19 @@
           <t>Structured JSON file fetcher</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>GET /api/v1/xapi/files/{id} and GET /api/v1/app/files/{id} return structured JSON (virtual quiz/assignments/attempts or stored files)</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Build the API</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2157,10 +2189,14 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I31" s="12" t="inlineStr"/>
+          <t>Fetch quiz JSON on Diagnostics xAPI tab</t>
+        </is>
+      </c>
+      <c r="I31" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2178,19 +2214,19 @@
           <t>Real-time grade sync from external modules</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Not implemented (inbound grades)</t>
+          <t>POST /api/v1/xapi/grades and POST /api/v1/app/grades ingest an external module score into quiz_attempts + xAPI; Moodle AGS stays outbound SoR</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Build the inbound grade endpoint</t>
+          <t>Inbound does not auto-AGS without an LTI launch</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2200,10 +2236,14 @@
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I32" s="12" t="inlineStr"/>
+          <t>Ingest grade control on Diagnostics xAPI tab</t>
+        </is>
+      </c>
+      <c r="I32" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2221,19 +2261,19 @@
           <t>Attempt counter synchronisation</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>GET /api/v1/xapi/attempts plus App API quota on /attempts; POST /attempts/sync merges an external used count with local graded attempts</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Build the endpoint</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2243,10 +2283,14 @@
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I33" s="12" t="inlineStr"/>
+          <t>Attempt counters on Diagnostics + Checkpoint</t>
+        </is>
+      </c>
+      <c r="I33" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2264,19 +2308,19 @@
           <t>Attempt limit enforcement</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Not implemented (no attempt limits in the quiz model)</t>
+          <t>Graded quiz GET returns quota; POST /quiz/submit 403 attempt_limit when used &gt;= max_attempts (default 3, teacher POST /quiz/policy)</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Add attempt limits</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2286,10 +2330,14 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I34" s="12" t="inlineStr"/>
+          <t>Live Attempt N of M on Checkpoint; submit blocked at the cap</t>
+        </is>
+      </c>
+      <c r="I34" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#quiz</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2354,19 +2402,19 @@
           <t>Universal file streamer (any file type)</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Files are served only for eBooks and specific exports</t>
+          <t>GET /files/{id}/stream on ops xAPI and App API streams PDF/MD/JSON/binary with detected Content-Type</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Build a general file streamer with access control</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2376,10 +2424,14 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I36" s="12" t="inlineStr"/>
+          <t>Stream assessment PDF on Diagnostics xAPI tab</t>
+        </is>
+      </c>
+      <c r="I36" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2397,19 +2449,19 @@
           <t>File type detection and routing</t>
         </is>
       </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>detect_file_kind sniffs extension, Content-Type, and magic bytes; /files/{id}/meta returns kind + json|stream route</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Build with F-9</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2419,10 +2471,14 @@
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I37" s="12" t="inlineStr"/>
+          <t>Detect PDF route on Diagnostics xAPI tab</t>
+        </is>
+      </c>
+      <c r="I37" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2440,19 +2496,19 @@
           <t>AI question bank from Technical Orders and uploads (20+ per document)</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>No Technical Order ingestion; AI draft from PDF exists but is not a TO bank</t>
+          <t>POST /api/v1/app/cat/bank drafts 20+ items from TO text or PDF/DOCX; SPA Checkpoint CAT generator; review then promote</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Build TO ingestion and bank generation</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2462,10 +2518,14 @@
       </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I38" s="12" t="inlineStr"/>
+          <t>Live 20+ TO question bank on Checkpoint</t>
+        </is>
+      </c>
+      <c r="I38" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#quiz</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2577,19 +2637,19 @@
           <t>AI competency mapper</t>
         </is>
       </c>
-      <c r="D41" s="11" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Implemented (code present)</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Competency maps come from a manually maintained skills registry, not AI extraction</t>
+          <t>POST /api/v1/app/cat/map extracts TO/EO/objective lines and matches or proposes skills; Diagnostics CAT mapper + proposal approve</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Build AI extraction from TOs</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2599,10 +2659,14 @@
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>Not started this phase</t>
-        </is>
-      </c>
-      <c r="I41" s="12" t="inlineStr"/>
+          <t>Live AI competency mapper on Diagnostics</t>
+        </is>
+      </c>
+      <c r="I41" s="14" t="inlineStr">
+        <is>
+          <t>https://edvidura-app-production.up.railway.app/app/#teacher-diagnostics</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4572,59 +4636,75 @@
   </sheetData>
   <autoFilter ref="A1:F84"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4684,13 +4764,13 @@
         <v>6</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -4706,13 +4786,13 @@
         <v>13</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -4728,13 +4808,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -4750,13 +4830,13 @@
         <v>10</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -4772,13 +4852,13 @@
         <v>4</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -4926,13 +5006,13 @@
         <v>83</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -5050,7 +5130,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>XR store, LTI groups, essay RAG, AR recorder, 100+ test bank, ML PLE</t>
+          <t>XR store, ML PLE, AR recorder, ADA checker, ETIMS, semantic search</t>
         </is>
       </c>
     </row>

</xml_diff>